<commit_message>
revision to plant protection
</commit_message>
<xml_diff>
--- a/docs/paper/eric_lychee_paper_submission.xlsx
+++ b/docs/paper/eric_lychee_paper_submission.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rzhuang/Documents/VscodeProjects/lychee/docs/paper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD7CC449-9033-B44B-AFA1-6000F250F5AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D8E2BBE-BC3F-D74E-AA74-7DF53E6DF10A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1060" yWindow="660" windowWidth="33500" windowHeight="21680" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="72">
   <si>
     <t>https://zenodo.org/records/22240717</t>
   </si>
@@ -244,6 +244,9 @@
   </si>
   <si>
     <t>MDPI plants</t>
+  </si>
+  <si>
+    <t>revised and submitted</t>
   </si>
 </sst>
 </file>
@@ -663,7 +666,7 @@
     <col min="3" max="3" width="21.1640625" style="11" customWidth="1"/>
     <col min="4" max="4" width="8.6640625" style="11" customWidth="1"/>
     <col min="5" max="5" width="7.83203125" style="11" customWidth="1"/>
-    <col min="6" max="6" width="12.6640625" style="11"/>
+    <col min="6" max="6" width="22.33203125" style="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="16" x14ac:dyDescent="0.2">
@@ -830,8 +833,11 @@
       <c r="E8" s="11">
         <v>1</v>
       </c>
+      <c r="F8" s="11" t="s">
+        <v>71</v>
+      </c>
       <c r="G8">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:23" ht="18" x14ac:dyDescent="0.2">

</xml_diff>